<commit_message>
adding AI python notes
</commit_message>
<xml_diff>
--- a/Cloud/Cloud_services.xlsx
+++ b/Cloud/Cloud_services.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Srinivasa Reddy B\Desktop\Seenu\Cloud\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Srinivasa Reddy B\Desktop\Github\Technologies\Cloud\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FC547AD-3767-4E63-8725-E6FFB0769696}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB37C48D-F9FB-4614-BF32-41E9B2D034C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="298" uniqueCount="291">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="309" uniqueCount="302">
   <si>
     <t>Developer Tools</t>
   </si>
@@ -910,6 +910,39 @@
   </si>
   <si>
     <t>Elastic Container Registry</t>
+  </si>
+  <si>
+    <t>Concepts to learn</t>
+  </si>
+  <si>
+    <t>Azure Service Connections</t>
+  </si>
+  <si>
+    <t>Pipeline Agents</t>
+  </si>
+  <si>
+    <t>Variable Groups</t>
+  </si>
+  <si>
+    <t>Environments</t>
+  </si>
+  <si>
+    <t>Release Gates</t>
+  </si>
+  <si>
+    <t>Multi-stage YAML pipelines</t>
+  </si>
+  <si>
+    <t>AKS deployments</t>
+  </si>
+  <si>
+    <t>Terraform with Azure DevOps</t>
+  </si>
+  <si>
+    <t>Key Vault integration</t>
+  </si>
+  <si>
+    <t>Self-hosted agents</t>
   </si>
 </sst>
 </file>
@@ -1005,14 +1038,12 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1020,9 +1051,11 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1400,7 +1433,7 @@
       <c r="D7" s="1" t="s">
         <v>192</v>
       </c>
-      <c r="E7" s="7"/>
+      <c r="E7" s="5"/>
       <c r="G7" s="1"/>
       <c r="H7" s="2" t="s">
         <v>259</v>
@@ -1412,7 +1445,7 @@
         <v>7</v>
       </c>
       <c r="D8" s="1"/>
-      <c r="E8" s="8" t="s">
+      <c r="E8" s="6" t="s">
         <v>193</v>
       </c>
       <c r="G8" s="1"/>
@@ -1426,7 +1459,7 @@
         <v>8</v>
       </c>
       <c r="D9" s="1"/>
-      <c r="E9" s="8" t="s">
+      <c r="E9" s="6" t="s">
         <v>194</v>
       </c>
       <c r="G9" s="1"/>
@@ -1440,7 +1473,7 @@
         <v>9</v>
       </c>
       <c r="D10" s="1"/>
-      <c r="E10" s="8" t="s">
+      <c r="E10" s="6" t="s">
         <v>195</v>
       </c>
       <c r="G10" s="1"/>
@@ -1454,7 +1487,7 @@
         <v>10</v>
       </c>
       <c r="D11" s="1"/>
-      <c r="E11" s="8" t="s">
+      <c r="E11" s="6" t="s">
         <v>196</v>
       </c>
       <c r="G11" s="1"/>
@@ -1468,7 +1501,7 @@
         <v>11</v>
       </c>
       <c r="D12" s="1"/>
-      <c r="E12" s="8" t="s">
+      <c r="E12" s="6" t="s">
         <v>197</v>
       </c>
     </row>
@@ -1478,7 +1511,7 @@
         <v>12</v>
       </c>
       <c r="D13" s="1"/>
-      <c r="E13" s="7" t="s">
+      <c r="E13" s="5" t="s">
         <v>198</v>
       </c>
       <c r="G13" s="1" t="s">
@@ -1492,7 +1525,7 @@
         <v>13</v>
       </c>
       <c r="D14" s="1"/>
-      <c r="E14" s="7" t="s">
+      <c r="E14" s="5" t="s">
         <v>199</v>
       </c>
       <c r="G14" s="1"/>
@@ -1506,7 +1539,7 @@
         <v>14</v>
       </c>
       <c r="D15" s="1"/>
-      <c r="E15" s="7" t="s">
+      <c r="E15" s="5" t="s">
         <v>200</v>
       </c>
       <c r="G15" s="1"/>
@@ -1516,7 +1549,7 @@
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="D16" s="1"/>
-      <c r="E16" s="8" t="s">
+      <c r="E16" s="6" t="s">
         <v>201</v>
       </c>
       <c r="G16" s="1"/>
@@ -2176,14 +2209,15 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{517DC8A6-BF04-41EA-80E3-A57CD96560E3}">
-  <dimension ref="A1:E85"/>
+  <dimension ref="A1:G85"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="32.33203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="32.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="25.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
         <v>43</v>
       </c>
@@ -2192,92 +2226,125 @@
         <v>122</v>
       </c>
       <c r="E1" s="9"/>
-    </row>
-    <row r="2" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B2" s="11" t="s">
+      <c r="G1" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B2" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="7" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B3" s="11" t="s">
+      <c r="G2" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B3" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" s="7" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G3" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B4" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="7" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G4" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B5" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" s="7" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G5" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B6" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="E6" s="7" t="s">
         <v>124</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G6" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B7" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="E7" s="7" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G7" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B8" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="E8" s="3" t="s">
+      <c r="E8" s="7" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B9" s="11" t="s">
+      <c r="G8" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B9" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="E9" s="3" t="s">
+      <c r="E9" s="7" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G9" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B10" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="E10" s="6" t="s">
+      <c r="E10" s="12" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G10" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B11" s="4" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G11" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B12" s="4"/>
       <c r="D12" s="9" t="s">
         <v>129</v>
       </c>
       <c r="E12" s="9"/>
     </row>
-    <row r="13" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A13" s="10" t="s">
         <v>54</v>
       </c>
@@ -2286,24 +2353,24 @@
         <v>130</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B14" s="11" t="s">
+    <row r="14" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B14" s="7" t="s">
         <v>55</v>
       </c>
       <c r="E14" s="3" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B15" s="11" t="s">
+    <row r="15" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B15" s="7" t="s">
         <v>56</v>
       </c>
       <c r="E15" s="3" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B16" s="11" t="s">
+    <row r="16" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B16" s="7" t="s">
         <v>57</v>
       </c>
       <c r="E16" s="3" t="s">
@@ -2311,7 +2378,7 @@
       </c>
     </row>
     <row r="17" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B17" s="11" t="s">
+      <c r="B17" s="7" t="s">
         <v>58</v>
       </c>
       <c r="E17" s="3" t="s">
@@ -2319,7 +2386,7 @@
       </c>
     </row>
     <row r="18" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B18" s="11" t="s">
+      <c r="B18" s="7" t="s">
         <v>59</v>
       </c>
       <c r="E18" s="3" t="s">
@@ -2327,7 +2394,7 @@
       </c>
     </row>
     <row r="19" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B19" s="11" t="s">
+      <c r="B19" s="7" t="s">
         <v>60</v>
       </c>
       <c r="E19" s="3" t="s">
@@ -2335,7 +2402,7 @@
       </c>
     </row>
     <row r="20" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B20" s="11" t="s">
+      <c r="B20" s="7" t="s">
         <v>61</v>
       </c>
       <c r="E20" s="3" t="s">
@@ -2343,12 +2410,12 @@
       </c>
     </row>
     <row r="21" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B21" s="11" t="s">
+      <c r="B21" s="7" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B22" s="11" t="s">
+      <c r="B22" s="7" t="s">
         <v>63</v>
       </c>
       <c r="D22" s="9" t="s">
@@ -2357,7 +2424,7 @@
       <c r="E22" s="9"/>
     </row>
     <row r="23" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B23" s="11" t="s">
+      <c r="B23" s="7" t="s">
         <v>64</v>
       </c>
       <c r="E23" s="3" t="s">
@@ -2365,7 +2432,7 @@
       </c>
     </row>
     <row r="24" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B24" s="11" t="s">
+      <c r="B24" s="7" t="s">
         <v>65</v>
       </c>
       <c r="E24" s="3" t="s">
@@ -2373,7 +2440,7 @@
       </c>
     </row>
     <row r="25" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B25" s="11" t="s">
+      <c r="B25" s="7" t="s">
         <v>66</v>
       </c>
       <c r="E25" s="3" t="s">
@@ -2381,7 +2448,7 @@
       </c>
     </row>
     <row r="26" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B26" s="11" t="s">
+      <c r="B26" s="7" t="s">
         <v>67</v>
       </c>
       <c r="E26" s="3" t="s">
@@ -2389,7 +2456,7 @@
       </c>
     </row>
     <row r="27" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B27" s="11" t="s">
+      <c r="B27" s="7" t="s">
         <v>68</v>
       </c>
       <c r="E27" s="3" t="s">
@@ -2397,7 +2464,7 @@
       </c>
     </row>
     <row r="28" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B28" s="11" t="s">
+      <c r="B28" s="7" t="s">
         <v>69</v>
       </c>
       <c r="E28" s="3" t="s">
@@ -2405,7 +2472,7 @@
       </c>
     </row>
     <row r="29" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B29" s="11" t="s">
+      <c r="B29" s="7" t="s">
         <v>70</v>
       </c>
       <c r="E29" s="3" t="s">
@@ -2413,7 +2480,7 @@
       </c>
     </row>
     <row r="30" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B30" s="12" t="s">
+      <c r="B30" s="8" t="s">
         <v>71</v>
       </c>
       <c r="E30" s="3" t="s">
@@ -2432,7 +2499,7 @@
       <c r="B32" s="9"/>
     </row>
     <row r="33" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B33" s="11" t="s">
+      <c r="B33" s="7" t="s">
         <v>73</v>
       </c>
       <c r="D33" s="9" t="s">
@@ -2441,7 +2508,7 @@
       <c r="E33" s="9"/>
     </row>
     <row r="34" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B34" s="11" t="s">
+      <c r="B34" s="7" t="s">
         <v>74</v>
       </c>
       <c r="E34" s="3" t="s">
@@ -2449,7 +2516,7 @@
       </c>
     </row>
     <row r="35" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B35" s="11" t="s">
+      <c r="B35" s="7" t="s">
         <v>75</v>
       </c>
       <c r="E35" s="3" t="s">
@@ -2457,7 +2524,7 @@
       </c>
     </row>
     <row r="36" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B36" s="11" t="s">
+      <c r="B36" s="7" t="s">
         <v>76</v>
       </c>
       <c r="E36" s="3" t="s">
@@ -2465,7 +2532,7 @@
       </c>
     </row>
     <row r="37" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B37" s="11" t="s">
+      <c r="B37" s="7" t="s">
         <v>77</v>
       </c>
       <c r="E37" s="3" t="s">
@@ -2473,7 +2540,7 @@
       </c>
     </row>
     <row r="38" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B38" s="11" t="s">
+      <c r="B38" s="7" t="s">
         <v>78</v>
       </c>
       <c r="E38" s="3" t="s">
@@ -2481,7 +2548,7 @@
       </c>
     </row>
     <row r="39" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B39" s="11" t="s">
+      <c r="B39" s="7" t="s">
         <v>79</v>
       </c>
       <c r="E39" s="4" t="s">
@@ -2489,7 +2556,7 @@
       </c>
     </row>
     <row r="40" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B40" s="11" t="s">
+      <c r="B40" s="7" t="s">
         <v>80</v>
       </c>
     </row>
@@ -2588,37 +2655,37 @@
       <c r="B55" s="9"/>
     </row>
     <row r="56" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B56" s="11" t="s">
+      <c r="B56" s="7" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="57" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B57" s="11" t="s">
+      <c r="B57" s="7" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="58" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B58" s="11" t="s">
+      <c r="B58" s="7" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="59" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B59" s="11" t="s">
+      <c r="B59" s="7" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="60" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B60" s="11" t="s">
+      <c r="B60" s="7" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="61" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B61" s="11" t="s">
+      <c r="B61" s="7" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="62" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B62" s="12" t="s">
+      <c r="B62" s="8" t="s">
         <v>100</v>
       </c>
     </row>
@@ -2675,57 +2742,57 @@
       <c r="B74" s="9"/>
     </row>
     <row r="75" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B75" s="3" t="s">
+      <c r="B75" s="7" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="76" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B76" s="5" t="s">
+      <c r="B76" s="11" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="77" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B77" s="5" t="s">
+      <c r="B77" s="11" t="s">
         <v>113</v>
       </c>
     </row>
     <row r="78" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B78" s="5" t="s">
+      <c r="B78" s="11" t="s">
         <v>114</v>
       </c>
     </row>
     <row r="79" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B79" s="5" t="s">
+      <c r="B79" s="11" t="s">
         <v>115</v>
       </c>
     </row>
     <row r="80" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B80" s="5" t="s">
+      <c r="B80" s="11" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="81" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B81" s="3" t="s">
+      <c r="B81" s="7" t="s">
         <v>117</v>
       </c>
     </row>
     <row r="82" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B82" s="3" t="s">
+      <c r="B82" s="7" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="83" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B83" s="3" t="s">
+      <c r="B83" s="7" t="s">
         <v>119</v>
       </c>
     </row>
     <row r="84" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B84" s="3" t="s">
+      <c r="B84" s="7" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="85" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B85" s="3" t="s">
+      <c r="B85" s="7" t="s">
         <v>121</v>
       </c>
     </row>

</xml_diff>